<commit_message>
fix: unblock build when RESEND_API_KEY is absent
Resend's constructor throws at module import if the key is undefined,
which breaks Next.js "Collecting page data" during build. The last two
deploys failed because of this — production has been stuck on 11-day-old
code, which is why the assessment 404 fix never shipped.

Fall back to a placeholder string when the env var is missing so modules
can load. Actual send() calls will still fail at runtime when the key is
truly misconfigured — that error should be surfaced, not swallowed.

Note: production needs RESEND_API_KEY set in Vercel env for emails to
actually send.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Rehab database/Business expense v1.xlsx
+++ b/Rehab database/Business expense v1.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29822"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="14" documentId="8_{071639FA-00AA-4128-B9F9-1BA9383A75D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{95E05B61-EAE7-4147-AF3C-AB5C35C31799}"/>
+  <xr:revisionPtr revIDLastSave="16" documentId="8_{071639FA-00AA-4128-B9F9-1BA9383A75D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{253AE081-392A-4C7C-937D-1647428CE1D8}"/>
   <bookViews>
-    <workbookView xWindow="-21697" yWindow="-98" windowWidth="21795" windowHeight="13875" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Expense Report" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="25">
   <si>
     <t>Sales</t>
   </si>
@@ -114,6 +114,9 @@
   </si>
   <si>
     <t>Vercel</t>
+  </si>
+  <si>
+    <t>Antropic API</t>
   </si>
 </sst>
 </file>
@@ -1095,7 +1098,13 @@
     </row>
     <row r="17" spans="2:6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B17" s="6"/>
-      <c r="E17" s="8"/>
+      <c r="D17" t="s">
+        <v>24</v>
+      </c>
+      <c r="E17" s="8">
+        <f>26.75*32</f>
+        <v>856</v>
+      </c>
       <c r="F17" s="8"/>
     </row>
     <row r="18" spans="2:6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -1126,7 +1135,7 @@
       <c r="D22" s="2"/>
       <c r="E22" s="3">
         <f>SUBTOTAL(109,Expenses[Amount])</f>
-        <v>11265.880000000001</v>
+        <v>12121.880000000001</v>
       </c>
       <c r="F22" s="3">
         <f>SUBTOTAL(109,Expenses[Remark])</f>
@@ -1187,6 +1196,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010079F111ED35F8CC479449609E8A0923A6" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="9677210f24a1be23c92c90fd886aa0aa">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5" xmlns:ns3="16c05727-aa75-4e4a-9b5f-8a80a1165891" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="60e05723c5c1908df1a1a4ebf11d344e" ns2:_="" ns3:_="">
     <xsd:import namespace="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5"/>
@@ -1397,15 +1415,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -1415,6 +1424,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C1564FA1-A819-4B0C-A3D7-4C70AEDB2621}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B5B48A48-5268-4115-B2F2-4BF9481F03B3}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1433,14 +1450,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C1564FA1-A819-4B0C-A3D7-4C70AEDB2621}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{169CA549-0B83-46B7-BE42-08D27B16AA2F}">
   <ds:schemaRefs>

</xml_diff>